<commit_message>
lost count of what is happening at this point
</commit_message>
<xml_diff>
--- a/data/human_datasheet_Kirill.xlsx
+++ b/data/human_datasheet_Kirill.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ender\OneDrive\Documents\Kirill\Uni\YEAR2\CSC211\csc211-env\verification-of-responses\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF9E970C-97E5-4D1D-A156-52DA928CA3CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DD05542-92EB-43CF-927A-BE14D5151594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,77 +28,77 @@
     <t>text</t>
   </si>
   <si>
-    <t>I'm not smoking while people use "wylie smokes too much" to justify ruining my shit</t>
-  </si>
-  <si>
-    <t>Account holder, this is the microsoft security team. There are security concerns on your account. To remain in good standing, follow the official steps to review your account today. Failure to respond may result in a hold. Regards, Cameron Nguyen</t>
-  </si>
-  <si>
-    <t>Yup but it's not giving me problems now so mayb i'll jus leave it...</t>
-  </si>
-  <si>
-    <t>Okï¿½beautiful..</t>
-  </si>
-  <si>
-    <t>Attention, your account requires verification. To restore access, reset your password and enter your username, 2FA verification code, and recovery key. Sincerely, Taylor Brown</t>
-  </si>
-  <si>
-    <t>Dear customer, your login has been restricted. Use the secure link to verify your username and restore access. Enter your username and password to continue. Security Team, Taylor Singh</t>
-  </si>
-  <si>
-    <t>Thanks for attending the workshop. Here are the links to references and the slide deck. Appreciate your feedback on this draft. Best, Casey Lee</t>
-  </si>
-  <si>
-    <t>Dear user, this is the facebook compliance team. There are security concerns on your account. To remain in good standing, follow the confidential steps to review your account today. Failure to respond may result in a suspension. Sincerely, Avery Brown</t>
-  </si>
-  <si>
-    <t>Aight, I should be there by 8 at the latest, probably closer to 7. Are jay and tyler down or should we just do two trips?</t>
-  </si>
-  <si>
-    <t>It could work, we'll reach a consensus at the next meeting</t>
-  </si>
-  <si>
-    <t>Attaching the draft proposal. Feedback by Friday would be appreciated so we can finalize for the client. I'll share the slides later today. Best, Jordan Khan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yes fine </t>
-  </si>
-  <si>
-    <t>Notice, you have a new notification. Please click here to view the update. For your convenience, a link and attachment are included. Do not reply to this auto-generated message. Security Team, Taylor Kim</t>
-  </si>
-  <si>
-    <t>The 2 oz guy is being kinda flaky but one friend is interested in picking up $ &amp;lt;#&amp;gt;  worth tonight if possible</t>
-  </si>
-  <si>
-    <t>Sharing the revised documentation with examples. The new endpoints are described in section two. Let me know if the timing works for you. Best, Taylor Kim</t>
-  </si>
-  <si>
-    <t>Hello, confirming our meeting on Thursday at 2 PM in the conference room. Please bring the draft slides for review. Let me know if the timing works for you. Best, Avery Nguyen</t>
-  </si>
-  <si>
-    <t>as a valued customer, i embody pleased to propose you that survey recent review of your mob no. you are awarded with a Â£1500 bonus prize, call 09066368470</t>
-  </si>
-  <si>
-    <t>Thanks for attending the workshop. Here are links to references and the slide deck. Let me know if the timing works for you. Best, Casey Wong</t>
-  </si>
-  <si>
-    <t>Hi there, congratulations! You are the winner of a prize. To redeem your payment of 3 BTC, please provide your account number to process the amount. This offer is limited time. Regards, Taylor Garcia</t>
-  </si>
-  <si>
-    <t>atm block:dear customer, due to our system promote your atm card has just been de-activated. to trigger call customer care 7679046492 now.</t>
+    <t xml:space="preserve">Dear V0DAF0NE Customer,You are a 5,00,000 winner of Guaranteed Caller Prize, this is our Final attempt to contact you! To Claim Call 7679046492 Now! </t>
+  </si>
+  <si>
+    <t>Have a great trip to India. And bring the light to everyone not just with the project but with everyone that is lucky to see you smile. Bye. Abiola</t>
+  </si>
+  <si>
+    <t>Its ok, if anybody asks abt me, u tel them..:-P</t>
+  </si>
+  <si>
+    <t>Account holder, congratulations! You are the winner of a prize. To claim your payment of $10,000, please provide your account number to process the sum. This offer is limited time. Sincerely, Sam Kim</t>
+  </si>
+  <si>
+    <t>rt-king pro video club&gt;&gt; need help? info@ringtoneking.co.uk or call 08701237397 you must exist 16+ club credits redeemable at www.ringtoneking.co.uk! enjoy!</t>
+  </si>
+  <si>
+    <t>recpt 1/3. you have say a ringtone. your order is being processed...</t>
+  </si>
+  <si>
+    <t>Why you Dint come with us.</t>
+  </si>
+  <si>
+    <t>Dear customer, you have a new notification. Please click here to view the update. For your convenience, a link and attachment are included. Do not reply to this auto-generated message. Compliance Team, Riley Khan</t>
+  </si>
+  <si>
+    <t>Your board is working fine. The issue of overheating is also reslove. But still software inst is pending. I will come around 8'o clock.</t>
+  </si>
+  <si>
+    <t>&amp;lt;#&amp;gt;  am I think? Should say on syllabus</t>
+  </si>
+  <si>
+    <t>What you doing?how are you? Hope everything is fine..</t>
+  </si>
+  <si>
+    <t>Dear user, the IT department detected a malware infection on your workstation. Run the antivirus scan and install the security patch from the provided link to fix the issue. IT Desk, Riley Brown</t>
+  </si>
+  <si>
+    <t>Dear customer, congratulations! You are the winner of a reward. To claim your payment of $10,000, please provide your account number to process the amount. This deal is available today only. Sincerely, Sam Lee</t>
+  </si>
+  <si>
+    <t>Hi, Mobile no. 7645092312 has added you in their contact list on www.fullonsms.com It s a great place to send free sms to people For more visit fullonsms.com</t>
+  </si>
+  <si>
+    <t>Dear customer, congratulations! You are the selected recipient of a prize. To collect your payment of Â£2,500, please provide your routing number to process the total. This deal is available today only. Compliance Team, Alex Wong</t>
+  </si>
+  <si>
+    <t>Please find the minutes from our last meeting. Action items are listed at the end of the note for convenience. Feel free to add notes before we meet. Best, Alex Brown</t>
+  </si>
+  <si>
+    <t>Last chance 2 claim ur å£150 worth of discount vouchers-Text YES to 85023 now!SavaMob-member offers mobile T Cs 08717898035. å£3.00 Sub. 16 . Remove txt X or STOP</t>
+  </si>
+  <si>
+    <t>loan for any purpose Â£500 - Â£75,000. homeowners + tenants welcome. possess you exist previously refused? we can still help. call free 0800 1956669 or text back 'help'</t>
+  </si>
+  <si>
+    <t>I booked the lab for next Wednesday. The calendar invite includes location and equipment details. I'll share the slides later today. Best, Jamie Wong</t>
+  </si>
+  <si>
+    <t>Attention, this is the apple security team. There are policy concerns on your account. To remain in good standing, follow the confidential steps to review your account today. Failure to respond may result in a hold. IT Desk, Morgan Lee</t>
+  </si>
+  <si>
+    <t>spam</t>
   </si>
   <si>
     <t>ham</t>
-  </si>
-  <si>
-    <t>spam</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -106,28 +106,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Arial"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF305496"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -142,11 +127,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -458,170 +442,170 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" s="2" t="s">
+    <row r="2" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="42" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B3" s="2" t="s">
+    <row r="3" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" s="2" t="s">
+      <c r="A4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="2" t="s">
+    <row r="5" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="28" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" s="2" t="s">
+    <row r="6" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="28" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" s="2" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="28" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" s="2" t="s">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="42" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B9" s="2" t="s">
+    <row r="9" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="28" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" s="2" t="s">
+    <row r="10" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="2" t="s">
+      <c r="A11" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="28" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="2" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="2" t="s">
+    <row r="13" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="28" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B14" s="2" t="s">
+    <row r="14" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A15" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B15" s="2" t="s">
+    <row r="15" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="28" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B16" s="2" t="s">
+    <row r="16" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="28" x14ac:dyDescent="0.35">
-      <c r="A17" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B17" s="2" t="s">
+    <row r="17" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="28" x14ac:dyDescent="0.35">
-      <c r="A18" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B18" s="2" t="s">
+    <row r="18" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="28" x14ac:dyDescent="0.35">
-      <c r="A19" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B19" s="2" t="s">
+    <row r="19" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A19" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="28" x14ac:dyDescent="0.35">
-      <c r="A20" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B20" s="2" t="s">
+    <row r="20" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="28" x14ac:dyDescent="0.35">
-      <c r="A21" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B21" s="2" t="s">
+    <row r="21" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A21" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>